<commit_message>
Atualizando dados do dashboard
</commit_message>
<xml_diff>
--- a/[CISSA] Relatório do Curso Ciber para Empreendedores.xlsx
+++ b/[CISSA] Relatório do Curso Ciber para Empreendedores.xlsx
@@ -136,7 +136,7 @@
       </c>
       <c r="G2" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H2" s="0" t="inlineStr">
@@ -178,7 +178,7 @@
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>74 dias 18 horas</t>
+          <t>81 dias 18 horas</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -200,7 +200,7 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>Ativo</t>
+          <t>Não atualmente</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
@@ -220,7 +220,7 @@
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>19 dias 23 horas</t>
+          <t>26 dias 23 horas</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -262,7 +262,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -346,7 +346,7 @@
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -388,7 +388,7 @@
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -430,7 +430,7 @@
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -472,7 +472,7 @@
       </c>
       <c r="G10" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H10" s="0" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="G11" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H11" s="0" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="G13" s="0" t="inlineStr">
         <is>
-          <t>82 dias 19 horas</t>
+          <t>89 dias 19 horas</t>
         </is>
       </c>
       <c r="H13" s="0" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="G14" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H14" s="0" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t>95 dias 23 horas</t>
+          <t>102 dias 23 horas</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="G16" s="0" t="inlineStr">
         <is>
-          <t>88 dias 22 horas</t>
+          <t>95 dias 22 horas</t>
         </is>
       </c>
       <c r="H16" s="0" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="G17" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H17" s="0" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t>66 dias 18 horas</t>
+          <t>73 dias 18 horas</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="G19" s="0" t="inlineStr">
         <is>
-          <t>74 dias 18 horas</t>
+          <t>81 dias 18 horas</t>
         </is>
       </c>
       <c r="H19" s="0" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="G20" s="0" t="inlineStr">
         <is>
-          <t>95 dias 23 horas</t>
+          <t>102 dias 23 horas</t>
         </is>
       </c>
       <c r="H20" s="0" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t>66 dias 18 horas</t>
+          <t>73 dias 18 horas</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="G22" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H22" s="0" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G23" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H23" s="0" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G25" s="0" t="inlineStr">
         <is>
-          <t>16 dias 18 horas</t>
+          <t>23 dias 18 horas</t>
         </is>
       </c>
       <c r="H25" s="0" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="G26" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H26" s="0" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G27" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H27" s="0" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G28" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H28" s="0" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="G29" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H29" s="0" t="inlineStr">
         <is>
-          <t>sexta-feira, 13 fev. 2026, 16:46</t>
+          <t>terça-feira, 31 mar. 2026, 09:22</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="G30" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H30" s="0" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="G33" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H33" s="0" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="G34" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H34" s="0" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="G35" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H35" s="0" t="inlineStr">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="G36" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H36" s="0" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="G37" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H37" s="0" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="G38" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H38" s="0" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="G39" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H39" s="0" t="inlineStr">
@@ -1707,12 +1707,12 @@
       </c>
       <c r="D40" s="0" t="inlineStr">
         <is>
-          <t>20,0%</t>
+          <t>100,0%</t>
         </is>
       </c>
       <c r="E40" s="0" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="G40" s="0" t="inlineStr">
@@ -1722,7 +1722,7 @@
       </c>
       <c r="H40" s="0" t="inlineStr">
         <is>
-          <t>segunda-feira, 9 mar. 2026, 21:06</t>
+          <t>segunda-feira, 30 mar. 2026, 15:42</t>
         </is>
       </c>
     </row>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="G41" s="0" t="inlineStr">
         <is>
-          <t>10 dias 16 horas</t>
+          <t>17 dias 16 horas</t>
         </is>
       </c>
       <c r="H41" s="0" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="G42" s="0" t="inlineStr">
         <is>
-          <t>67 dias 18 horas</t>
+          <t>74 dias 18 horas</t>
         </is>
       </c>
       <c r="H42" s="0" t="inlineStr">
@@ -1843,7 +1843,7 @@
       </c>
       <c r="G43" s="0" t="inlineStr">
         <is>
-          <t>61 dias 18 horas</t>
+          <t>68 dias 18 horas</t>
         </is>
       </c>
       <c r="H43" s="0" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="G44" s="0" t="inlineStr">
         <is>
-          <t>66 dias 18 horas</t>
+          <t>73 dias 18 horas</t>
         </is>
       </c>
       <c r="H44" s="0" t="inlineStr">

</xml_diff>